<commit_message>
updated erdbeer & verkostung ergebnis
</commit_message>
<xml_diff>
--- a/data/gold/Erdbeer Clustering Sensorik Vorgabe.xlsx
+++ b/data/gold/Erdbeer Clustering Sensorik Vorgabe.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\Aroma\Flavor Development\Portfolio Management\K_AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778402C7-1F48-4827-B405-D09413959092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1D5515-4FAE-4FB3-A93E-436FB223837C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{41210865-F3E7-4CFB-AA9B-77A6475D37BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="111">
   <si>
     <t>Deskriptoren allgemein</t>
   </si>
@@ -326,9 +326,6 @@
     <t>187.800</t>
   </si>
   <si>
-    <t>187.916</t>
-  </si>
-  <si>
     <t>187.894</t>
   </si>
   <si>
@@ -338,9 +335,6 @@
     <t>185.267</t>
   </si>
   <si>
-    <t>186.521</t>
-  </si>
-  <si>
     <t>wenn Rohstoff vorhanden</t>
   </si>
   <si>
@@ -375,6 +369,9 @@
   </si>
   <si>
     <t>&gt; 0,1 eindeutig</t>
+  </si>
+  <si>
+    <t>187.772</t>
   </si>
 </sst>
 </file>
@@ -419,7 +416,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -765,11 +762,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -802,6 +838,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1136,7 +1176,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7D75154-37C5-4E01-94B7-8DDFF36C29F1}">
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.6328125" customWidth="1"/>
@@ -1145,8 +1185,8 @@
     <col min="5" max="5" width="15.81640625" customWidth="1"/>
     <col min="7" max="7" width="11.1796875" customWidth="1"/>
     <col min="8" max="8" width="14.81640625" customWidth="1"/>
-    <col min="9" max="9" width="24.26953125" customWidth="1"/>
-    <col min="10" max="10" width="21.26953125" customWidth="1"/>
+    <col min="9" max="9" width="24.1796875" customWidth="1"/>
+    <col min="10" max="10" width="21.1796875" customWidth="1"/>
     <col min="11" max="11" width="24.36328125" customWidth="1"/>
     <col min="12" max="12" width="22.6328125" customWidth="1"/>
     <col min="13" max="13" width="12.90625" customWidth="1"/>
@@ -1155,7 +1195,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1279,61 +1319,81 @@
       </c>
       <c r="N3" s="17"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
+    <row r="4" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5"/>
       <c r="B4" s="10" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7" t="s">
+      <c r="E4" s="34"/>
+      <c r="F4" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="34">
         <v>0.4884</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="34">
         <v>63</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="34">
         <v>3.1729E-2</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="34">
         <v>1.5495E-2</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="34">
         <v>8.3099999999999997E-3</v>
       </c>
-      <c r="L4" s="7">
+      <c r="L4" s="34">
         <v>0</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="M4" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="N4" s="17"/>
+      <c r="N4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="5"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="N5" s="20"/>
+      <c r="A5" s="32"/>
+      <c r="B5" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" s="21"/>
+      <c r="F5" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" s="21">
+        <v>0.1085</v>
+      </c>
+      <c r="H5" s="21">
+        <v>14</v>
+      </c>
+      <c r="I5" s="21">
+        <v>1.0430000000000001E-3</v>
+      </c>
+      <c r="J5" s="21">
+        <v>1.13E-4</v>
+      </c>
+      <c r="K5" s="21">
+        <v>4.7699999999999999E-4</v>
+      </c>
+      <c r="L5" s="21">
+        <v>0</v>
+      </c>
+      <c r="M5" s="21"/>
+      <c r="N5" s="24" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="6" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="28" t="s">
@@ -1372,7 +1432,7 @@
       </c>
       <c r="M6" s="21"/>
       <c r="N6" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -1413,10 +1473,10 @@
         <v>0</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1494,7 +1554,7 @@
         <v>88</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -1613,10 +1673,10 @@
         <v>0</v>
       </c>
       <c r="M12" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1695,273 +1755,225 @@
         <v>7.5989999999999999E-3</v>
       </c>
       <c r="M14" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="N14" s="16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="19" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="24"/>
+    </row>
+    <row r="20" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20" s="14">
+        <v>3.8800000000000001E-2</v>
+      </c>
+      <c r="H20" s="14">
+        <v>5</v>
+      </c>
+      <c r="I20" s="14">
+        <v>1.402E-3</v>
+      </c>
+      <c r="J20" s="14">
+        <v>5.3999999999999998E-5</v>
+      </c>
+      <c r="K20" s="14">
+        <v>7.7999999999999999E-5</v>
+      </c>
+      <c r="L20" s="14">
+        <v>0</v>
+      </c>
+      <c r="M20" s="14"/>
+      <c r="N20" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="N14" s="16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="5"/>
-      <c r="B15" s="26"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="N15" s="20"/>
-    </row>
-    <row r="16" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="28"/>
-      <c r="B16" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="E16" s="21"/>
-      <c r="F16" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="G16" s="21">
-        <v>0.1085</v>
-      </c>
-      <c r="H16" s="21">
-        <v>14</v>
-      </c>
-      <c r="I16" s="21">
-        <v>1.0430000000000001E-3</v>
-      </c>
-      <c r="J16" s="21">
-        <v>1.13E-4</v>
-      </c>
-      <c r="K16" s="21">
-        <v>4.7699999999999999E-4</v>
-      </c>
-      <c r="L16" s="21">
+    </row>
+    <row r="21" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="18"/>
+      <c r="B21" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="G21" s="19">
+        <v>7.7999999999999996E-3</v>
+      </c>
+      <c r="H21" s="19">
+        <v>1</v>
+      </c>
+      <c r="I21" s="19">
+        <v>9.4509999999999993E-3</v>
+      </c>
+      <c r="J21" s="19">
+        <v>7.2999999999999999E-5</v>
+      </c>
+      <c r="K21" s="19">
+        <v>9.4509999999999993E-3</v>
+      </c>
+      <c r="L21" s="19">
         <v>0</v>
       </c>
-      <c r="M16" s="21"/>
-      <c r="N16" s="24" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="21" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="24"/>
-    </row>
-    <row r="22" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M21" s="19"/>
+      <c r="N21" s="20"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="13" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G22" s="14">
-        <v>3.8800000000000001E-2</v>
+        <v>3.1E-2</v>
       </c>
       <c r="H22" s="14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I22" s="14">
-        <v>1.402E-3</v>
+        <v>1.1429999999999999E-3</v>
       </c>
       <c r="J22" s="14">
-        <v>5.3999999999999998E-5</v>
+        <v>3.4999999999999997E-5</v>
       </c>
       <c r="K22" s="14">
-        <v>7.7999999999999999E-5</v>
+        <v>4.86E-4</v>
       </c>
       <c r="L22" s="14">
         <v>0</v>
       </c>
-      <c r="M22" s="14"/>
-      <c r="N22" s="31" t="s">
-        <v>100</v>
+      <c r="M22" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="N22" s="16" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="18"/>
       <c r="B23" s="19" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
       <c r="F23" s="19" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="G23" s="19">
-        <v>7.7999999999999996E-3</v>
+        <v>0.21709999999999999</v>
       </c>
       <c r="H23" s="19">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="I23" s="19">
-        <v>9.4509999999999993E-3</v>
+        <v>2.6714000000000002E-2</v>
       </c>
       <c r="J23" s="19">
-        <v>7.2999999999999999E-5</v>
+        <v>5.7980000000000002E-3</v>
       </c>
       <c r="K23" s="19">
-        <v>9.4509999999999993E-3</v>
+        <v>3.9459999999999999E-3</v>
       </c>
       <c r="L23" s="19">
         <v>0</v>
       </c>
-      <c r="M23" s="19"/>
-      <c r="N23" s="20"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A24" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="G24" s="14">
-        <v>3.1E-2</v>
-      </c>
-      <c r="H24" s="14">
-        <v>4</v>
-      </c>
-      <c r="I24" s="14">
-        <v>1.1429999999999999E-3</v>
-      </c>
-      <c r="J24" s="14">
-        <v>3.4999999999999997E-5</v>
-      </c>
-      <c r="K24" s="14">
-        <v>4.86E-4</v>
-      </c>
-      <c r="L24" s="14">
+      <c r="M23" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="N23" s="20" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="G24" s="30">
+        <v>7.7999999999999996E-3</v>
+      </c>
+      <c r="H24" s="30">
+        <v>1</v>
+      </c>
+      <c r="I24" s="30">
+        <v>7.9999999999999996E-6</v>
+      </c>
+      <c r="J24" s="30">
         <v>0</v>
       </c>
-      <c r="M24" s="14" t="s">
+      <c r="K24" s="30">
+        <v>7.9999999999999996E-6</v>
+      </c>
+      <c r="L24" s="30">
+        <v>0</v>
+      </c>
+      <c r="M24" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="N24" s="16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="18"/>
-      <c r="B25" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="G25" s="19">
-        <v>0.21709999999999999</v>
-      </c>
-      <c r="H25" s="19">
+      <c r="N24" s="31" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="E30">
+        <f>7*4</f>
         <v>28</v>
-      </c>
-      <c r="I25" s="19">
-        <v>2.6714000000000002E-2</v>
-      </c>
-      <c r="J25" s="19">
-        <v>5.7980000000000002E-3</v>
-      </c>
-      <c r="K25" s="19">
-        <v>3.9459999999999999E-3</v>
-      </c>
-      <c r="L25" s="19">
-        <v>0</v>
-      </c>
-      <c r="M25" s="19"/>
-      <c r="N25" s="20" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="29" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="30" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="G26" s="30">
-        <v>7.7999999999999996E-3</v>
-      </c>
-      <c r="H26" s="30">
-        <v>1</v>
-      </c>
-      <c r="I26" s="30">
-        <v>7.9999999999999996E-6</v>
-      </c>
-      <c r="J26" s="30">
-        <v>0</v>
-      </c>
-      <c r="K26" s="30">
-        <v>7.9999999999999996E-6</v>
-      </c>
-      <c r="L26" s="30">
-        <v>0</v>
-      </c>
-      <c r="M26" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="N26" s="31" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>